<commit_message>
Atualização automática — 29/07/2026 15:29
</commit_message>
<xml_diff>
--- a/dados/dados_documentacao.xlsx
+++ b/dados/dados_documentacao.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5613" uniqueCount="1791">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5613" uniqueCount="1797">
   <si>
     <t>UF</t>
   </si>
@@ -5353,16 +5353,22 @@
     <t>Afastado</t>
   </si>
   <si>
+    <t>GISELE CHIOVATTO</t>
+  </si>
+  <si>
+    <t>PEDRO GUILHERME CRISPIM DOS ANJOS</t>
+  </si>
+  <si>
     <t>Não informado</t>
   </si>
   <si>
-    <t>PEDRO GUILHERME CRISPIM DOS ANJOS</t>
+    <t>THAYLA RAMALHO SILVA MACHADO</t>
   </si>
   <si>
     <t>FERNANDO KELLER SANTOS DE BRITO</t>
   </si>
   <si>
-    <t>THAYLA RAMALHO SILVA MACHADO</t>
+    <t>GISELE  MUNIZ SILVESTRE</t>
   </si>
   <si>
     <t>DILCINEIA BATISTA</t>
@@ -5371,19 +5377,31 @@
     <t>RODRIGO ALMEIDA DA COSTA</t>
   </si>
   <si>
+    <t>ENCONTRAR SUPERVISOR</t>
+  </si>
+  <si>
+    <t>NARCELIO RAMOS SOUZA</t>
+  </si>
+  <si>
     <t>RENATA MELO FERREIRA FELIX</t>
   </si>
   <si>
-    <t>NARCELIO RAMOS SOUZA</t>
+    <t>DEBORA JULIANA FERREIRA DA SILVA</t>
   </si>
   <si>
     <t>EDSON LOUZADA DOS ANJOS JUNIOR</t>
   </si>
   <si>
+    <t>JOAO DA CRUZ SANTOS</t>
+  </si>
+  <si>
+    <t>RAIANE LEAL PERCU</t>
+  </si>
+  <si>
     <t>GILNEI CASTRO</t>
   </si>
   <si>
-    <t>RAIANE LEAL PERCU</t>
+    <t>GILIARDE DE ANDRADE</t>
   </si>
   <si>
     <t>RONALD HENRIQUE DE OLIVEIRA MALTA</t>
@@ -5966,7 +5984,7 @@
         <v>1775</v>
       </c>
       <c r="X3" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -6040,7 +6058,7 @@
         <v>1776</v>
       </c>
       <c r="X4" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="5" spans="1:24">
@@ -6188,7 +6206,7 @@
         <v>1775</v>
       </c>
       <c r="X6" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:24">
@@ -6262,7 +6280,7 @@
         <v>1776</v>
       </c>
       <c r="X7" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="8" spans="1:24">
@@ -6336,7 +6354,7 @@
         <v>1775</v>
       </c>
       <c r="X8" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:24">
@@ -6410,7 +6428,7 @@
         <v>1775</v>
       </c>
       <c r="X9" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:24">
@@ -6484,7 +6502,7 @@
         <v>1775</v>
       </c>
       <c r="X10" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="11" spans="1:24">
@@ -6558,7 +6576,7 @@
         <v>1775</v>
       </c>
       <c r="X11" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="12" spans="1:24">
@@ -6706,7 +6724,7 @@
         <v>1777</v>
       </c>
       <c r="X13" t="s">
-        <v>1781</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="14" spans="1:24">
@@ -6854,7 +6872,7 @@
         <v>1775</v>
       </c>
       <c r="X15" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="16" spans="1:24">
@@ -7002,7 +7020,7 @@
         <v>1776</v>
       </c>
       <c r="X17" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="18" spans="1:24">
@@ -7076,7 +7094,7 @@
         <v>1775</v>
       </c>
       <c r="X18" t="s">
-        <v>1779</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="19" spans="1:24">
@@ -7224,7 +7242,7 @@
         <v>1776</v>
       </c>
       <c r="X20" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="21" spans="1:24">
@@ -7298,7 +7316,7 @@
         <v>1775</v>
       </c>
       <c r="X21" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="22" spans="1:24">
@@ -7446,7 +7464,7 @@
         <v>1776</v>
       </c>
       <c r="X23" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="24" spans="1:24">
@@ -7520,7 +7538,7 @@
         <v>1776</v>
       </c>
       <c r="X24" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="25" spans="1:24">
@@ -7594,7 +7612,7 @@
         <v>1776</v>
       </c>
       <c r="X25" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="26" spans="1:24">
@@ -7668,7 +7686,7 @@
         <v>1776</v>
       </c>
       <c r="X26" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="27" spans="1:24">
@@ -7742,7 +7760,7 @@
         <v>1775</v>
       </c>
       <c r="X27" t="s">
-        <v>1779</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="28" spans="1:24">
@@ -7890,7 +7908,7 @@
         <v>1776</v>
       </c>
       <c r="X29" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="30" spans="1:24">
@@ -7964,7 +7982,7 @@
         <v>1776</v>
       </c>
       <c r="X30" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="31" spans="1:24">
@@ -8038,7 +8056,7 @@
         <v>1776</v>
       </c>
       <c r="X31" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="32" spans="1:24">
@@ -8112,7 +8130,7 @@
         <v>1776</v>
       </c>
       <c r="X32" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="33" spans="1:24">
@@ -8186,7 +8204,7 @@
         <v>1775</v>
       </c>
       <c r="X33" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="34" spans="1:24">
@@ -8260,7 +8278,7 @@
         <v>1775</v>
       </c>
       <c r="X34" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="35" spans="1:24">
@@ -8408,7 +8426,7 @@
         <v>1776</v>
       </c>
       <c r="X36" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="37" spans="1:24">
@@ -8482,7 +8500,7 @@
         <v>1775</v>
       </c>
       <c r="X37" t="s">
-        <v>1779</v>
+        <v>69</v>
       </c>
     </row>
     <row r="38" spans="1:24">
@@ -8556,7 +8574,7 @@
         <v>1776</v>
       </c>
       <c r="X38" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="39" spans="1:24">
@@ -8630,7 +8648,7 @@
         <v>1776</v>
       </c>
       <c r="X39" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="40" spans="1:24">
@@ -8704,7 +8722,7 @@
         <v>1776</v>
       </c>
       <c r="X40" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="41" spans="1:24">
@@ -8852,7 +8870,7 @@
         <v>1775</v>
       </c>
       <c r="X42" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="43" spans="1:24">
@@ -8926,7 +8944,7 @@
         <v>1776</v>
       </c>
       <c r="X43" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="44" spans="1:24">
@@ -9000,7 +9018,7 @@
         <v>1775</v>
       </c>
       <c r="X44" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="45" spans="1:24">
@@ -9074,7 +9092,7 @@
         <v>1775</v>
       </c>
       <c r="X45" t="s">
-        <v>1779</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46" spans="1:24">
@@ -9148,7 +9166,7 @@
         <v>1775</v>
       </c>
       <c r="X46" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="47" spans="1:24">
@@ -9222,7 +9240,7 @@
         <v>1776</v>
       </c>
       <c r="X47" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="48" spans="1:24">
@@ -9296,7 +9314,7 @@
         <v>1778</v>
       </c>
       <c r="X48" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="49" spans="1:24">
@@ -9370,7 +9388,7 @@
         <v>1775</v>
       </c>
       <c r="X49" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="50" spans="1:24">
@@ -9444,7 +9462,7 @@
         <v>1776</v>
       </c>
       <c r="X50" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="51" spans="1:24">
@@ -9666,7 +9684,7 @@
         <v>1775</v>
       </c>
       <c r="X53" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="54" spans="1:24">
@@ -9740,7 +9758,7 @@
         <v>1776</v>
       </c>
       <c r="X54" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="55" spans="1:24">
@@ -9885,7 +9903,7 @@
         <v>1776</v>
       </c>
       <c r="X56" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="57" spans="1:24">
@@ -9959,7 +9977,7 @@
         <v>1775</v>
       </c>
       <c r="X57" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="58" spans="1:24">
@@ -10033,7 +10051,7 @@
         <v>1775</v>
       </c>
       <c r="X58" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="59" spans="1:24">
@@ -10107,7 +10125,7 @@
         <v>1775</v>
       </c>
       <c r="X59" t="s">
-        <v>1779</v>
+        <v>69</v>
       </c>
     </row>
     <row r="60" spans="1:24">
@@ -10255,7 +10273,7 @@
         <v>1776</v>
       </c>
       <c r="X61" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="62" spans="1:24">
@@ -10403,7 +10421,7 @@
         <v>1776</v>
       </c>
       <c r="X63" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="64" spans="1:24">
@@ -10477,7 +10495,7 @@
         <v>1776</v>
       </c>
       <c r="X64" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="65" spans="1:24">
@@ -10551,7 +10569,7 @@
         <v>1775</v>
       </c>
       <c r="X65" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="66" spans="1:24">
@@ -10696,7 +10714,7 @@
         <v>1775</v>
       </c>
       <c r="X67" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="68" spans="1:24">
@@ -10844,7 +10862,7 @@
         <v>1775</v>
       </c>
       <c r="X69" t="s">
-        <v>1779</v>
+        <v>69</v>
       </c>
     </row>
     <row r="70" spans="1:24">
@@ -10915,7 +10933,7 @@
         <v>1775</v>
       </c>
       <c r="X70" t="s">
-        <v>1779</v>
+        <v>69</v>
       </c>
     </row>
     <row r="71" spans="1:24">
@@ -10986,7 +11004,7 @@
         <v>1776</v>
       </c>
       <c r="X71" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="72" spans="1:24">
@@ -11134,7 +11152,7 @@
         <v>1776</v>
       </c>
       <c r="X73" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="74" spans="1:24">
@@ -11205,7 +11223,7 @@
         <v>1775</v>
       </c>
       <c r="X74" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="75" spans="1:24">
@@ -11279,7 +11297,7 @@
         <v>1777</v>
       </c>
       <c r="X75" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="76" spans="1:24">
@@ -11353,7 +11371,7 @@
         <v>1776</v>
       </c>
       <c r="X76" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="77" spans="1:24">
@@ -11427,7 +11445,7 @@
         <v>1776</v>
       </c>
       <c r="X77" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="78" spans="1:24">
@@ -11501,7 +11519,7 @@
         <v>1775</v>
       </c>
       <c r="X78" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="79" spans="1:24">
@@ -11575,7 +11593,7 @@
         <v>1776</v>
       </c>
       <c r="X79" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="80" spans="1:24">
@@ -11649,7 +11667,7 @@
         <v>1776</v>
       </c>
       <c r="X80" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="81" spans="1:24">
@@ -11723,7 +11741,7 @@
         <v>1775</v>
       </c>
       <c r="X81" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="82" spans="1:24">
@@ -11797,7 +11815,7 @@
         <v>1776</v>
       </c>
       <c r="X82" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="83" spans="1:24">
@@ -11871,7 +11889,7 @@
         <v>1775</v>
       </c>
       <c r="X83" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="84" spans="1:24">
@@ -11945,7 +11963,7 @@
         <v>1775</v>
       </c>
       <c r="X84" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="85" spans="1:24">
@@ -12019,7 +12037,7 @@
         <v>1776</v>
       </c>
       <c r="X85" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="86" spans="1:24">
@@ -12093,7 +12111,7 @@
         <v>1775</v>
       </c>
       <c r="X86" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="87" spans="1:24">
@@ -12167,7 +12185,7 @@
         <v>1777</v>
       </c>
       <c r="X87" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="88" spans="1:24">
@@ -12241,7 +12259,7 @@
         <v>1776</v>
       </c>
       <c r="X88" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="89" spans="1:24">
@@ -12315,7 +12333,7 @@
         <v>1775</v>
       </c>
       <c r="X89" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="90" spans="1:24">
@@ -12389,7 +12407,7 @@
         <v>1778</v>
       </c>
       <c r="X90" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="91" spans="1:24">
@@ -12463,7 +12481,7 @@
         <v>1777</v>
       </c>
       <c r="X91" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="92" spans="1:24">
@@ -12537,7 +12555,7 @@
         <v>1776</v>
       </c>
       <c r="X92" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="93" spans="1:24">
@@ -12611,7 +12629,7 @@
         <v>1775</v>
       </c>
       <c r="X93" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="94" spans="1:24">
@@ -12685,7 +12703,7 @@
         <v>1777</v>
       </c>
       <c r="X94" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="95" spans="1:24">
@@ -12759,7 +12777,7 @@
         <v>1776</v>
       </c>
       <c r="X95" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="96" spans="1:24">
@@ -12833,7 +12851,7 @@
         <v>1775</v>
       </c>
       <c r="X96" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="97" spans="1:24">
@@ -12907,7 +12925,7 @@
         <v>1775</v>
       </c>
       <c r="X97" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="98" spans="1:24">
@@ -12981,7 +12999,7 @@
         <v>1777</v>
       </c>
       <c r="X98" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="99" spans="1:24">
@@ -13055,7 +13073,7 @@
         <v>1777</v>
       </c>
       <c r="X99" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="100" spans="1:24">
@@ -13129,7 +13147,7 @@
         <v>1777</v>
       </c>
       <c r="X100" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="101" spans="1:24">
@@ -13203,7 +13221,7 @@
         <v>1776</v>
       </c>
       <c r="X101" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="102" spans="1:24">
@@ -13277,7 +13295,7 @@
         <v>1777</v>
       </c>
       <c r="X102" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="103" spans="1:24">
@@ -13351,7 +13369,7 @@
         <v>1778</v>
       </c>
       <c r="X103" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="104" spans="1:24">
@@ -13425,7 +13443,7 @@
         <v>1775</v>
       </c>
       <c r="X104" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="105" spans="1:24">
@@ -13499,7 +13517,7 @@
         <v>1776</v>
       </c>
       <c r="X105" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="106" spans="1:24">
@@ -13573,7 +13591,7 @@
         <v>1775</v>
       </c>
       <c r="X106" t="s">
-        <v>1779</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="107" spans="1:24">
@@ -13647,7 +13665,7 @@
         <v>1775</v>
       </c>
       <c r="X107" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="108" spans="1:24">
@@ -13721,7 +13739,7 @@
         <v>1777</v>
       </c>
       <c r="X108" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="109" spans="1:24">
@@ -13795,7 +13813,7 @@
         <v>1777</v>
       </c>
       <c r="X109" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="110" spans="1:24">
@@ -13869,7 +13887,7 @@
         <v>1776</v>
       </c>
       <c r="X110" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="111" spans="1:24">
@@ -13943,7 +13961,7 @@
         <v>1776</v>
       </c>
       <c r="X111" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="112" spans="1:24">
@@ -14017,7 +14035,7 @@
         <v>1775</v>
       </c>
       <c r="X112" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="113" spans="1:24">
@@ -14091,7 +14109,7 @@
         <v>1777</v>
       </c>
       <c r="X113" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="114" spans="1:24">
@@ -14165,7 +14183,7 @@
         <v>1777</v>
       </c>
       <c r="X114" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="115" spans="1:24">
@@ -14239,7 +14257,7 @@
         <v>1775</v>
       </c>
       <c r="X115" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="116" spans="1:24">
@@ -14313,7 +14331,7 @@
         <v>1778</v>
       </c>
       <c r="X116" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="117" spans="1:24">
@@ -14387,7 +14405,7 @@
         <v>1777</v>
       </c>
       <c r="X117" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="118" spans="1:24">
@@ -14461,7 +14479,7 @@
         <v>1777</v>
       </c>
       <c r="X118" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="119" spans="1:24">
@@ -14535,7 +14553,7 @@
         <v>1776</v>
       </c>
       <c r="X119" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="120" spans="1:24">
@@ -14683,7 +14701,7 @@
         <v>1775</v>
       </c>
       <c r="X121" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="122" spans="1:24">
@@ -14757,7 +14775,7 @@
         <v>1776</v>
       </c>
       <c r="X122" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="123" spans="1:24">
@@ -14831,7 +14849,7 @@
         <v>1775</v>
       </c>
       <c r="X123" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="124" spans="1:24">
@@ -14905,7 +14923,7 @@
         <v>1776</v>
       </c>
       <c r="X124" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="125" spans="1:24">
@@ -14979,7 +14997,7 @@
         <v>1775</v>
       </c>
       <c r="X125" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="126" spans="1:24">
@@ -15124,7 +15142,7 @@
         <v>1775</v>
       </c>
       <c r="X127" t="s">
-        <v>1779</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="128" spans="1:24">
@@ -15198,7 +15216,7 @@
         <v>1775</v>
       </c>
       <c r="X128" t="s">
-        <v>1779</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="129" spans="1:24">
@@ -15272,7 +15290,7 @@
         <v>1775</v>
       </c>
       <c r="X129" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="130" spans="1:24">
@@ -15346,7 +15364,7 @@
         <v>1776</v>
       </c>
       <c r="X130" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="131" spans="1:24">
@@ -15420,7 +15438,7 @@
         <v>1775</v>
       </c>
       <c r="X131" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="132" spans="1:24">
@@ -15494,7 +15512,7 @@
         <v>1775</v>
       </c>
       <c r="X132" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="133" spans="1:24">
@@ -15642,7 +15660,7 @@
         <v>1775</v>
       </c>
       <c r="X134" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="135" spans="1:24">
@@ -15790,7 +15808,7 @@
         <v>1775</v>
       </c>
       <c r="X136" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="137" spans="1:24">
@@ -16083,7 +16101,7 @@
         <v>1776</v>
       </c>
       <c r="X140" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="141" spans="1:24">
@@ -16157,7 +16175,7 @@
         <v>1775</v>
       </c>
       <c r="X141" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="142" spans="1:24">
@@ -16231,7 +16249,7 @@
         <v>1775</v>
       </c>
       <c r="X142" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="143" spans="1:24">
@@ -16379,7 +16397,7 @@
         <v>1775</v>
       </c>
       <c r="X144" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="145" spans="1:24">
@@ -16453,7 +16471,7 @@
         <v>1775</v>
       </c>
       <c r="X145" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="146" spans="1:24">
@@ -16527,7 +16545,7 @@
         <v>1775</v>
       </c>
       <c r="X146" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="147" spans="1:24">
@@ -16675,7 +16693,7 @@
         <v>1776</v>
       </c>
       <c r="X148" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="149" spans="1:24">
@@ -16823,7 +16841,7 @@
         <v>1775</v>
       </c>
       <c r="X150" t="s">
-        <v>1779</v>
+        <v>69</v>
       </c>
     </row>
     <row r="151" spans="1:24">
@@ -16897,7 +16915,7 @@
         <v>1776</v>
       </c>
       <c r="X151" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="152" spans="1:24">
@@ -16971,7 +16989,7 @@
         <v>1775</v>
       </c>
       <c r="X152" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="153" spans="1:24">
@@ -17045,7 +17063,7 @@
         <v>1775</v>
       </c>
       <c r="X153" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="154" spans="1:24">
@@ -17193,7 +17211,7 @@
         <v>1776</v>
       </c>
       <c r="X155" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="156" spans="1:24">
@@ -17267,7 +17285,7 @@
         <v>1776</v>
       </c>
       <c r="X156" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="157" spans="1:24">
@@ -17489,7 +17507,7 @@
         <v>1775</v>
       </c>
       <c r="X159" t="s">
-        <v>1779</v>
+        <v>69</v>
       </c>
     </row>
     <row r="160" spans="1:24">
@@ -17563,7 +17581,7 @@
         <v>1775</v>
       </c>
       <c r="X160" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="161" spans="1:24">
@@ -17637,7 +17655,7 @@
         <v>1775</v>
       </c>
       <c r="X161" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="162" spans="1:24">
@@ -17711,7 +17729,7 @@
         <v>1776</v>
       </c>
       <c r="X162" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="163" spans="1:24">
@@ -17859,7 +17877,7 @@
         <v>1776</v>
       </c>
       <c r="X164" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="165" spans="1:24">
@@ -17933,7 +17951,7 @@
         <v>1776</v>
       </c>
       <c r="X165" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="166" spans="1:24">
@@ -18081,7 +18099,7 @@
         <v>1775</v>
       </c>
       <c r="X167" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="168" spans="1:24">
@@ -18155,7 +18173,7 @@
         <v>1775</v>
       </c>
       <c r="X168" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="169" spans="1:24">
@@ -18229,7 +18247,7 @@
         <v>1775</v>
       </c>
       <c r="X169" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="170" spans="1:24">
@@ -18525,7 +18543,7 @@
         <v>1776</v>
       </c>
       <c r="X173" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="174" spans="1:24">
@@ -18599,7 +18617,7 @@
         <v>1775</v>
       </c>
       <c r="X174" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="175" spans="1:24">
@@ -18747,7 +18765,7 @@
         <v>1776</v>
       </c>
       <c r="X176" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="177" spans="1:24">
@@ -18821,7 +18839,7 @@
         <v>1776</v>
       </c>
       <c r="X177" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="178" spans="1:24">
@@ -18969,7 +18987,7 @@
         <v>1775</v>
       </c>
       <c r="X179" t="s">
-        <v>1779</v>
+        <v>69</v>
       </c>
     </row>
     <row r="180" spans="1:24">
@@ -19043,7 +19061,7 @@
         <v>1775</v>
       </c>
       <c r="X180" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="181" spans="1:24">
@@ -19117,7 +19135,7 @@
         <v>1775</v>
       </c>
       <c r="X181" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="182" spans="1:24">
@@ -19265,7 +19283,7 @@
         <v>1775</v>
       </c>
       <c r="X183" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="184" spans="1:24">
@@ -19339,7 +19357,7 @@
         <v>1775</v>
       </c>
       <c r="X184" t="s">
-        <v>1779</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="185" spans="1:24">
@@ -19487,7 +19505,7 @@
         <v>1775</v>
       </c>
       <c r="X186" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="187" spans="1:24">
@@ -19561,7 +19579,7 @@
         <v>1775</v>
       </c>
       <c r="X187" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="188" spans="1:24">
@@ -19709,7 +19727,7 @@
         <v>1775</v>
       </c>
       <c r="X189" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="190" spans="1:24">
@@ -19783,7 +19801,7 @@
         <v>1776</v>
       </c>
       <c r="X190" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="191" spans="1:24">
@@ -19857,7 +19875,7 @@
         <v>1775</v>
       </c>
       <c r="X191" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="192" spans="1:24">
@@ -20005,7 +20023,7 @@
         <v>1776</v>
       </c>
       <c r="X193" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="194" spans="1:24">
@@ -20079,7 +20097,7 @@
         <v>1776</v>
       </c>
       <c r="X194" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="195" spans="1:24">
@@ -20153,7 +20171,7 @@
         <v>1776</v>
       </c>
       <c r="X195" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="196" spans="1:24">
@@ -20449,7 +20467,7 @@
         <v>1775</v>
       </c>
       <c r="X199" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="200" spans="1:24">
@@ -20523,7 +20541,7 @@
         <v>1775</v>
       </c>
       <c r="X200" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="201" spans="1:24">
@@ -20597,7 +20615,7 @@
         <v>1775</v>
       </c>
       <c r="X201" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="202" spans="1:24">
@@ -20671,7 +20689,7 @@
         <v>1775</v>
       </c>
       <c r="X202" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="203" spans="1:24">
@@ -20745,7 +20763,7 @@
         <v>1776</v>
       </c>
       <c r="X203" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="204" spans="1:24">
@@ -20893,7 +20911,7 @@
         <v>1775</v>
       </c>
       <c r="X205" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="206" spans="1:24">
@@ -21041,7 +21059,7 @@
         <v>1778</v>
       </c>
       <c r="X207" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="208" spans="1:24">
@@ -21115,7 +21133,7 @@
         <v>1776</v>
       </c>
       <c r="X208" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="209" spans="1:24">
@@ -21189,7 +21207,7 @@
         <v>1775</v>
       </c>
       <c r="X209" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="210" spans="1:24">
@@ -21263,7 +21281,7 @@
         <v>1776</v>
       </c>
       <c r="X210" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="211" spans="1:24">
@@ -21337,7 +21355,7 @@
         <v>1775</v>
       </c>
       <c r="X211" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="212" spans="1:24">
@@ -21411,7 +21429,7 @@
         <v>1776</v>
       </c>
       <c r="X212" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="213" spans="1:24">
@@ -21485,7 +21503,7 @@
         <v>1776</v>
       </c>
       <c r="X213" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="214" spans="1:24">
@@ -21633,7 +21651,7 @@
         <v>1775</v>
       </c>
       <c r="X215" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="216" spans="1:24">
@@ -21781,7 +21799,7 @@
         <v>1775</v>
       </c>
       <c r="X217" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="218" spans="1:24">
@@ -21855,7 +21873,7 @@
         <v>1775</v>
       </c>
       <c r="X218" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="219" spans="1:24">
@@ -21929,7 +21947,7 @@
         <v>1776</v>
       </c>
       <c r="X219" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="220" spans="1:24">
@@ -22003,7 +22021,7 @@
         <v>1775</v>
       </c>
       <c r="X220" t="s">
-        <v>1779</v>
+        <v>80</v>
       </c>
     </row>
     <row r="221" spans="1:24">
@@ -22077,7 +22095,7 @@
         <v>1776</v>
       </c>
       <c r="X221" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="222" spans="1:24">
@@ -22148,7 +22166,7 @@
         <v>1776</v>
       </c>
       <c r="X222" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="223" spans="1:24">
@@ -22222,7 +22240,7 @@
         <v>1775</v>
       </c>
       <c r="X223" t="s">
-        <v>1779</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="224" spans="1:24">
@@ -22296,7 +22314,7 @@
         <v>1777</v>
       </c>
       <c r="X224" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="225" spans="1:24">
@@ -22370,7 +22388,7 @@
         <v>1777</v>
       </c>
       <c r="X225" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="226" spans="1:24">
@@ -22444,7 +22462,7 @@
         <v>1775</v>
       </c>
       <c r="X226" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="227" spans="1:24">
@@ -22518,7 +22536,7 @@
         <v>1777</v>
       </c>
       <c r="X227" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="228" spans="1:24">
@@ -22592,7 +22610,7 @@
         <v>1776</v>
       </c>
       <c r="X228" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="229" spans="1:24">
@@ -22666,7 +22684,7 @@
         <v>1775</v>
       </c>
       <c r="X229" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="230" spans="1:24">
@@ -22740,7 +22758,7 @@
         <v>1776</v>
       </c>
       <c r="X230" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="231" spans="1:24">
@@ -22814,7 +22832,7 @@
         <v>1777</v>
       </c>
       <c r="X231" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="232" spans="1:24">
@@ -22888,7 +22906,7 @@
         <v>1777</v>
       </c>
       <c r="X232" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="233" spans="1:24">
@@ -22962,7 +22980,7 @@
         <v>1775</v>
       </c>
       <c r="X233" t="s">
-        <v>1779</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="234" spans="1:24">
@@ -23036,7 +23054,7 @@
         <v>1775</v>
       </c>
       <c r="X234" t="s">
-        <v>1779</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="235" spans="1:24">
@@ -23110,7 +23128,7 @@
         <v>1777</v>
       </c>
       <c r="X235" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="236" spans="1:24">
@@ -23184,7 +23202,7 @@
         <v>1777</v>
       </c>
       <c r="X236" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="237" spans="1:24">
@@ -23258,7 +23276,7 @@
         <v>1777</v>
       </c>
       <c r="X237" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="238" spans="1:24">
@@ -23332,7 +23350,7 @@
         <v>1777</v>
       </c>
       <c r="X238" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="239" spans="1:24">
@@ -23406,7 +23424,7 @@
         <v>1776</v>
       </c>
       <c r="X239" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="240" spans="1:24">
@@ -23480,7 +23498,7 @@
         <v>1776</v>
       </c>
       <c r="X240" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="241" spans="1:24">
@@ -23554,7 +23572,7 @@
         <v>1776</v>
       </c>
       <c r="X241" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="242" spans="1:24">
@@ -23628,7 +23646,7 @@
         <v>1776</v>
       </c>
       <c r="X242" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="243" spans="1:24">
@@ -23702,7 +23720,7 @@
         <v>1778</v>
       </c>
       <c r="X243" t="s">
-        <v>1779</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="244" spans="1:24">
@@ -23776,7 +23794,7 @@
         <v>1777</v>
       </c>
       <c r="X244" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="245" spans="1:24">
@@ -23850,7 +23868,7 @@
         <v>1775</v>
       </c>
       <c r="X245" t="s">
-        <v>1779</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="246" spans="1:24">
@@ -23924,7 +23942,7 @@
         <v>1777</v>
       </c>
       <c r="X246" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="247" spans="1:24">
@@ -23998,7 +24016,7 @@
         <v>1777</v>
       </c>
       <c r="X247" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="248" spans="1:24">
@@ -24072,7 +24090,7 @@
         <v>1777</v>
       </c>
       <c r="X248" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="249" spans="1:24">
@@ -24146,7 +24164,7 @@
         <v>1775</v>
       </c>
       <c r="X249" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="250" spans="1:24">
@@ -24220,7 +24238,7 @@
         <v>1777</v>
       </c>
       <c r="X250" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="251" spans="1:24">
@@ -24294,7 +24312,7 @@
         <v>1775</v>
       </c>
       <c r="X251" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="252" spans="1:24">
@@ -24368,7 +24386,7 @@
         <v>1777</v>
       </c>
       <c r="X252" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="253" spans="1:24">
@@ -24442,7 +24460,7 @@
         <v>1775</v>
       </c>
       <c r="X253" t="s">
-        <v>1779</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="254" spans="1:24">
@@ -24516,7 +24534,7 @@
         <v>1777</v>
       </c>
       <c r="X254" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="255" spans="1:24">
@@ -24590,7 +24608,7 @@
         <v>1777</v>
       </c>
       <c r="X255" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="256" spans="1:24">
@@ -24664,7 +24682,7 @@
         <v>1777</v>
       </c>
       <c r="X256" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="257" spans="1:24">
@@ -24738,7 +24756,7 @@
         <v>1777</v>
       </c>
       <c r="X257" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="258" spans="1:24">
@@ -24812,7 +24830,7 @@
         <v>1776</v>
       </c>
       <c r="X258" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="259" spans="1:24">
@@ -24886,7 +24904,7 @@
         <v>1777</v>
       </c>
       <c r="X259" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="260" spans="1:24">
@@ -24960,7 +24978,7 @@
         <v>1776</v>
       </c>
       <c r="X260" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="261" spans="1:24">
@@ -25034,7 +25052,7 @@
         <v>1775</v>
       </c>
       <c r="X261" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="262" spans="1:24">
@@ -25108,7 +25126,7 @@
         <v>1775</v>
       </c>
       <c r="X262" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="263" spans="1:24">
@@ -25182,7 +25200,7 @@
         <v>1777</v>
       </c>
       <c r="X263" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="264" spans="1:24">
@@ -25256,7 +25274,7 @@
         <v>1776</v>
       </c>
       <c r="X264" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="265" spans="1:24">
@@ -25330,7 +25348,7 @@
         <v>1776</v>
       </c>
       <c r="X265" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="266" spans="1:24">
@@ -25404,7 +25422,7 @@
         <v>1776</v>
       </c>
       <c r="X266" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="267" spans="1:24">
@@ -25478,7 +25496,7 @@
         <v>1777</v>
       </c>
       <c r="X267" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="268" spans="1:24">
@@ -25552,7 +25570,7 @@
         <v>1777</v>
       </c>
       <c r="X268" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="269" spans="1:24">
@@ -25626,7 +25644,7 @@
         <v>1777</v>
       </c>
       <c r="X269" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="270" spans="1:24">
@@ -25700,7 +25718,7 @@
         <v>1776</v>
       </c>
       <c r="X270" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="271" spans="1:24">
@@ -25774,7 +25792,7 @@
         <v>1777</v>
       </c>
       <c r="X271" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="272" spans="1:24">
@@ -25848,7 +25866,7 @@
         <v>1777</v>
       </c>
       <c r="X272" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="273" spans="1:24">
@@ -25922,7 +25940,7 @@
         <v>1775</v>
       </c>
       <c r="X273" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="274" spans="1:24">
@@ -25996,7 +26014,7 @@
         <v>1777</v>
       </c>
       <c r="X274" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="275" spans="1:24">
@@ -26070,7 +26088,7 @@
         <v>1775</v>
       </c>
       <c r="X275" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="276" spans="1:24">
@@ -26144,7 +26162,7 @@
         <v>1775</v>
       </c>
       <c r="X276" t="s">
-        <v>1779</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="277" spans="1:24">
@@ -26218,7 +26236,7 @@
         <v>1775</v>
       </c>
       <c r="X277" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="278" spans="1:24">
@@ -26292,7 +26310,7 @@
         <v>1775</v>
       </c>
       <c r="X278" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="279" spans="1:24">
@@ -26366,7 +26384,7 @@
         <v>1775</v>
       </c>
       <c r="X279" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="280" spans="1:24">
@@ -26440,7 +26458,7 @@
         <v>1776</v>
       </c>
       <c r="X280" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="281" spans="1:24">
@@ -26514,7 +26532,7 @@
         <v>1777</v>
       </c>
       <c r="X281" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="282" spans="1:24">
@@ -26588,7 +26606,7 @@
         <v>1775</v>
       </c>
       <c r="X282" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="283" spans="1:24">
@@ -26662,7 +26680,7 @@
         <v>1776</v>
       </c>
       <c r="X283" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="284" spans="1:24">
@@ -26736,7 +26754,7 @@
         <v>1777</v>
       </c>
       <c r="X284" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="285" spans="1:24">
@@ -26810,7 +26828,7 @@
         <v>1777</v>
       </c>
       <c r="X285" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="286" spans="1:24">
@@ -26884,7 +26902,7 @@
         <v>1777</v>
       </c>
       <c r="X286" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="287" spans="1:24">
@@ -26958,7 +26976,7 @@
         <v>1776</v>
       </c>
       <c r="X287" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="288" spans="1:24">
@@ -27032,7 +27050,7 @@
         <v>1775</v>
       </c>
       <c r="X288" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="289" spans="1:24">
@@ -27106,7 +27124,7 @@
         <v>1777</v>
       </c>
       <c r="X289" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="290" spans="1:24">
@@ -27180,7 +27198,7 @@
         <v>1776</v>
       </c>
       <c r="X290" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="291" spans="1:24">
@@ -27254,7 +27272,7 @@
         <v>1775</v>
       </c>
       <c r="X291" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="292" spans="1:24">
@@ -27328,7 +27346,7 @@
         <v>1777</v>
       </c>
       <c r="X292" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="293" spans="1:24">
@@ -27402,7 +27420,7 @@
         <v>1777</v>
       </c>
       <c r="X293" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="294" spans="1:24">
@@ -27473,7 +27491,7 @@
         <v>1777</v>
       </c>
       <c r="X294" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="295" spans="1:24">
@@ -27547,7 +27565,7 @@
         <v>1776</v>
       </c>
       <c r="X295" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="296" spans="1:24">
@@ -27621,7 +27639,7 @@
         <v>1777</v>
       </c>
       <c r="X296" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="297" spans="1:24">
@@ -27695,7 +27713,7 @@
         <v>1777</v>
       </c>
       <c r="X297" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="298" spans="1:24">
@@ -27769,7 +27787,7 @@
         <v>1775</v>
       </c>
       <c r="X298" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="299" spans="1:24">
@@ -27843,7 +27861,7 @@
         <v>1777</v>
       </c>
       <c r="X299" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="300" spans="1:24">
@@ -27917,7 +27935,7 @@
         <v>1777</v>
       </c>
       <c r="X300" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="301" spans="1:24">
@@ -27991,7 +28009,7 @@
         <v>1775</v>
       </c>
       <c r="X301" t="s">
-        <v>1779</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="302" spans="1:24">
@@ -28065,7 +28083,7 @@
         <v>1777</v>
       </c>
       <c r="X302" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="303" spans="1:24">
@@ -28139,7 +28157,7 @@
         <v>1775</v>
       </c>
       <c r="X303" t="s">
-        <v>1779</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="304" spans="1:24">
@@ -28213,7 +28231,7 @@
         <v>1776</v>
       </c>
       <c r="X304" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="305" spans="1:24">
@@ -28287,7 +28305,7 @@
         <v>1777</v>
       </c>
       <c r="X305" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="306" spans="1:24">
@@ -28361,7 +28379,7 @@
         <v>1777</v>
       </c>
       <c r="X306" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="307" spans="1:24">
@@ -28435,7 +28453,7 @@
         <v>1777</v>
       </c>
       <c r="X307" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="308" spans="1:24">
@@ -28509,7 +28527,7 @@
         <v>1777</v>
       </c>
       <c r="X308" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="309" spans="1:24">
@@ -28583,7 +28601,7 @@
         <v>1776</v>
       </c>
       <c r="X309" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="310" spans="1:24">
@@ -28657,7 +28675,7 @@
         <v>1775</v>
       </c>
       <c r="X310" t="s">
-        <v>1779</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="311" spans="1:24">
@@ -28731,7 +28749,7 @@
         <v>1777</v>
       </c>
       <c r="X311" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="312" spans="1:24">
@@ -28805,7 +28823,7 @@
         <v>1775</v>
       </c>
       <c r="X312" t="s">
-        <v>1779</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="313" spans="1:24">
@@ -28879,7 +28897,7 @@
         <v>1777</v>
       </c>
       <c r="X313" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="314" spans="1:24">
@@ -28953,7 +28971,7 @@
         <v>1777</v>
       </c>
       <c r="X314" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="315" spans="1:24">
@@ -29027,7 +29045,7 @@
         <v>1777</v>
       </c>
       <c r="X315" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="316" spans="1:24">
@@ -29101,7 +29119,7 @@
         <v>1777</v>
       </c>
       <c r="X316" t="s">
-        <v>1785</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="317" spans="1:24">
@@ -29175,7 +29193,7 @@
         <v>1775</v>
       </c>
       <c r="X317" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="318" spans="1:24">
@@ -29249,7 +29267,7 @@
         <v>1777</v>
       </c>
       <c r="X318" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="319" spans="1:24">
@@ -29323,7 +29341,7 @@
         <v>1776</v>
       </c>
       <c r="X319" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="320" spans="1:24">
@@ -29397,7 +29415,7 @@
         <v>1777</v>
       </c>
       <c r="X320" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="321" spans="1:24">
@@ -29471,7 +29489,7 @@
         <v>1777</v>
       </c>
       <c r="X321" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="322" spans="1:24">
@@ -29545,7 +29563,7 @@
         <v>1775</v>
       </c>
       <c r="X322" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="323" spans="1:24">
@@ -29619,7 +29637,7 @@
         <v>1777</v>
       </c>
       <c r="X323" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="324" spans="1:24">
@@ -29767,7 +29785,7 @@
         <v>1775</v>
       </c>
       <c r="X325" t="s">
-        <v>1779</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="326" spans="1:24">
@@ -29841,7 +29859,7 @@
         <v>1777</v>
       </c>
       <c r="X326" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="327" spans="1:24">
@@ -29915,7 +29933,7 @@
         <v>1775</v>
       </c>
       <c r="X327" t="s">
-        <v>1779</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="328" spans="1:24">
@@ -29989,7 +30007,7 @@
         <v>1775</v>
       </c>
       <c r="X328" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="329" spans="1:24">
@@ -30063,7 +30081,7 @@
         <v>1776</v>
       </c>
       <c r="X329" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="330" spans="1:24">
@@ -30137,7 +30155,7 @@
         <v>1776</v>
       </c>
       <c r="X330" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="331" spans="1:24">
@@ -30211,7 +30229,7 @@
         <v>1775</v>
       </c>
       <c r="X331" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="332" spans="1:24">
@@ -30285,7 +30303,7 @@
         <v>1776</v>
       </c>
       <c r="X332" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="333" spans="1:24">
@@ -30359,7 +30377,7 @@
         <v>1776</v>
       </c>
       <c r="X333" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="334" spans="1:24">
@@ -30433,7 +30451,7 @@
         <v>1776</v>
       </c>
       <c r="X334" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="335" spans="1:24">
@@ -30507,7 +30525,7 @@
         <v>1776</v>
       </c>
       <c r="X335" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="336" spans="1:24">
@@ -30581,7 +30599,7 @@
         <v>1776</v>
       </c>
       <c r="X336" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="337" spans="1:24">
@@ -30655,7 +30673,7 @@
         <v>1776</v>
       </c>
       <c r="X337" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="338" spans="1:24">
@@ -30729,7 +30747,7 @@
         <v>1775</v>
       </c>
       <c r="X338" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="339" spans="1:24">
@@ -30803,7 +30821,7 @@
         <v>1776</v>
       </c>
       <c r="X339" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="340" spans="1:24">
@@ -30874,7 +30892,7 @@
         <v>1777</v>
       </c>
       <c r="X340" t="s">
-        <v>1788</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="341" spans="1:24">
@@ -30948,7 +30966,7 @@
         <v>1775</v>
       </c>
       <c r="X341" t="s">
-        <v>1779</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="342" spans="1:24">
@@ -31022,7 +31040,7 @@
         <v>1775</v>
       </c>
       <c r="X342" t="s">
-        <v>1779</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="343" spans="1:24">
@@ -31096,7 +31114,7 @@
         <v>1776</v>
       </c>
       <c r="X343" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="344" spans="1:24">
@@ -31170,7 +31188,7 @@
         <v>1775</v>
       </c>
       <c r="X344" t="s">
-        <v>1779</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="345" spans="1:24">
@@ -31244,7 +31262,7 @@
         <v>1775</v>
       </c>
       <c r="X345" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="346" spans="1:24">
@@ -31392,7 +31410,7 @@
         <v>1775</v>
       </c>
       <c r="X347" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="348" spans="1:24">
@@ -31614,7 +31632,7 @@
         <v>1775</v>
       </c>
       <c r="X350" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="351" spans="1:24">
@@ -31836,7 +31854,7 @@
         <v>1776</v>
       </c>
       <c r="X353" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="354" spans="1:24">
@@ -32058,7 +32076,7 @@
         <v>1777</v>
       </c>
       <c r="X356" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="357" spans="1:24">
@@ -32132,7 +32150,7 @@
         <v>1775</v>
       </c>
       <c r="X357" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="358" spans="1:24">
@@ -32280,7 +32298,7 @@
         <v>1775</v>
       </c>
       <c r="X359" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="360" spans="1:24">
@@ -32354,7 +32372,7 @@
         <v>1775</v>
       </c>
       <c r="X360" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="361" spans="1:24">
@@ -32576,7 +32594,7 @@
         <v>1775</v>
       </c>
       <c r="X363" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="364" spans="1:24">
@@ -32724,7 +32742,7 @@
         <v>1775</v>
       </c>
       <c r="X365" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="366" spans="1:24">
@@ -32946,7 +32964,7 @@
         <v>1776</v>
       </c>
       <c r="X368" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="369" spans="1:24">
@@ -33020,7 +33038,7 @@
         <v>1775</v>
       </c>
       <c r="X369" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="370" spans="1:24">
@@ -33094,7 +33112,7 @@
         <v>1776</v>
       </c>
       <c r="X370" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="371" spans="1:24">
@@ -33168,7 +33186,7 @@
         <v>1776</v>
       </c>
       <c r="X371" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="372" spans="1:24">
@@ -33242,7 +33260,7 @@
         <v>1775</v>
       </c>
       <c r="X372" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="373" spans="1:24">
@@ -33316,7 +33334,7 @@
         <v>1775</v>
       </c>
       <c r="X373" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="374" spans="1:24">
@@ -33390,7 +33408,7 @@
         <v>1775</v>
       </c>
       <c r="X374" t="s">
-        <v>1779</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="375" spans="1:24">
@@ -33538,7 +33556,7 @@
         <v>1775</v>
       </c>
       <c r="X376" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="377" spans="1:24">
@@ -33612,7 +33630,7 @@
         <v>1775</v>
       </c>
       <c r="X377" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="378" spans="1:24">
@@ -33760,7 +33778,7 @@
         <v>1777</v>
       </c>
       <c r="X379" t="s">
-        <v>1781</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="380" spans="1:24">
@@ -33834,7 +33852,7 @@
         <v>1775</v>
       </c>
       <c r="X380" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="381" spans="1:24">
@@ -33982,7 +34000,7 @@
         <v>1775</v>
       </c>
       <c r="X382" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="383" spans="1:24">
@@ -34130,7 +34148,7 @@
         <v>1775</v>
       </c>
       <c r="X384" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="385" spans="1:24">
@@ -34204,7 +34222,7 @@
         <v>1776</v>
       </c>
       <c r="X385" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="386" spans="1:24">
@@ -34278,7 +34296,7 @@
         <v>1775</v>
       </c>
       <c r="X386" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="387" spans="1:24">
@@ -34352,7 +34370,7 @@
         <v>1775</v>
       </c>
       <c r="X387" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="388" spans="1:24">
@@ -34574,7 +34592,7 @@
         <v>1775</v>
       </c>
       <c r="X390" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="391" spans="1:24">
@@ -34722,7 +34740,7 @@
         <v>1776</v>
       </c>
       <c r="X392" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="393" spans="1:24">
@@ -34870,7 +34888,7 @@
         <v>1776</v>
       </c>
       <c r="X394" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="395" spans="1:24">
@@ -34944,7 +34962,7 @@
         <v>1775</v>
       </c>
       <c r="X395" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="396" spans="1:24">
@@ -35018,7 +35036,7 @@
         <v>1775</v>
       </c>
       <c r="X396" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="397" spans="1:24">
@@ -35092,7 +35110,7 @@
         <v>1775</v>
       </c>
       <c r="X397" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="398" spans="1:24">
@@ -35166,7 +35184,7 @@
         <v>1775</v>
       </c>
       <c r="X398" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="399" spans="1:24">
@@ -35240,7 +35258,7 @@
         <v>1778</v>
       </c>
       <c r="X399" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="400" spans="1:24">
@@ -35536,7 +35554,7 @@
         <v>1776</v>
       </c>
       <c r="X403" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="404" spans="1:24">
@@ -35607,7 +35625,7 @@
         <v>1775</v>
       </c>
       <c r="X404" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="405" spans="1:24">
@@ -35681,7 +35699,7 @@
         <v>1775</v>
       </c>
       <c r="X405" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="406" spans="1:24">
@@ -35755,7 +35773,7 @@
         <v>1775</v>
       </c>
       <c r="X406" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="407" spans="1:24">
@@ -35829,7 +35847,7 @@
         <v>1775</v>
       </c>
       <c r="X407" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="408" spans="1:24">
@@ -35903,7 +35921,7 @@
         <v>1775</v>
       </c>
       <c r="X408" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="409" spans="1:24">
@@ -36273,7 +36291,7 @@
         <v>1776</v>
       </c>
       <c r="X413" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="414" spans="1:24">
@@ -36347,7 +36365,7 @@
         <v>1775</v>
       </c>
       <c r="X414" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="415" spans="1:24">
@@ -36421,7 +36439,7 @@
         <v>1775</v>
       </c>
       <c r="X415" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="416" spans="1:24">
@@ -36495,7 +36513,7 @@
         <v>1775</v>
       </c>
       <c r="X416" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="417" spans="1:24">
@@ -36637,7 +36655,7 @@
         <v>1776</v>
       </c>
       <c r="X418" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="419" spans="1:24">
@@ -36711,7 +36729,7 @@
         <v>1776</v>
       </c>
       <c r="X419" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="420" spans="1:24">
@@ -36782,7 +36800,7 @@
         <v>1775</v>
       </c>
       <c r="X420" t="s">
-        <v>1779</v>
+        <v>441</v>
       </c>
     </row>
     <row r="421" spans="1:24">
@@ -36856,7 +36874,7 @@
         <v>1776</v>
       </c>
       <c r="X421" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="422" spans="1:24">
@@ -36930,7 +36948,7 @@
         <v>1777</v>
       </c>
       <c r="X422" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="423" spans="1:24">
@@ -37004,7 +37022,7 @@
         <v>1777</v>
       </c>
       <c r="X423" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="424" spans="1:24">
@@ -37078,7 +37096,7 @@
         <v>1777</v>
       </c>
       <c r="X424" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="425" spans="1:24">
@@ -37152,7 +37170,7 @@
         <v>1777</v>
       </c>
       <c r="X425" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="426" spans="1:24">
@@ -37226,7 +37244,7 @@
         <v>1777</v>
       </c>
       <c r="X426" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="427" spans="1:24">
@@ -37297,7 +37315,7 @@
         <v>1775</v>
       </c>
       <c r="X427" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="428" spans="1:24">
@@ -37371,7 +37389,7 @@
         <v>1777</v>
       </c>
       <c r="X428" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="429" spans="1:24">
@@ -37445,7 +37463,7 @@
         <v>1775</v>
       </c>
       <c r="X429" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="430" spans="1:24">
@@ -37519,7 +37537,7 @@
         <v>1775</v>
       </c>
       <c r="X430" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="431" spans="1:24">
@@ -37593,7 +37611,7 @@
         <v>1777</v>
       </c>
       <c r="X431" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="432" spans="1:24">
@@ -37667,7 +37685,7 @@
         <v>1775</v>
       </c>
       <c r="X432" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="433" spans="1:24">
@@ -37741,7 +37759,7 @@
         <v>1777</v>
       </c>
       <c r="X433" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="434" spans="1:24">
@@ -37815,7 +37833,7 @@
         <v>1775</v>
       </c>
       <c r="X434" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="435" spans="1:24">
@@ -37889,7 +37907,7 @@
         <v>1776</v>
       </c>
       <c r="X435" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="436" spans="1:24">
@@ -37963,7 +37981,7 @@
         <v>1775</v>
       </c>
       <c r="X436" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="437" spans="1:24">
@@ -38037,7 +38055,7 @@
         <v>1776</v>
       </c>
       <c r="X437" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="438" spans="1:24">
@@ -38111,7 +38129,7 @@
         <v>1775</v>
       </c>
       <c r="X438" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="439" spans="1:24">
@@ -38185,7 +38203,7 @@
         <v>1775</v>
       </c>
       <c r="X439" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="440" spans="1:24">
@@ -38259,7 +38277,7 @@
         <v>1775</v>
       </c>
       <c r="X440" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="441" spans="1:24">
@@ -38333,7 +38351,7 @@
         <v>1777</v>
       </c>
       <c r="X441" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="442" spans="1:24">
@@ -38407,7 +38425,7 @@
         <v>1777</v>
       </c>
       <c r="X442" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="443" spans="1:24">
@@ -38481,7 +38499,7 @@
         <v>1777</v>
       </c>
       <c r="X443" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="444" spans="1:24">
@@ -38555,7 +38573,7 @@
         <v>1777</v>
       </c>
       <c r="X444" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="445" spans="1:24">
@@ -38629,7 +38647,7 @@
         <v>1775</v>
       </c>
       <c r="X445" t="s">
-        <v>1779</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="446" spans="1:24">
@@ -38703,7 +38721,7 @@
         <v>1775</v>
       </c>
       <c r="X446" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="447" spans="1:24">
@@ -38777,7 +38795,7 @@
         <v>1777</v>
       </c>
       <c r="X447" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="448" spans="1:24">
@@ -38851,7 +38869,7 @@
         <v>1775</v>
       </c>
       <c r="X448" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="449" spans="1:24">
@@ -38925,7 +38943,7 @@
         <v>1776</v>
       </c>
       <c r="X449" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="450" spans="1:24">
@@ -38996,7 +39014,7 @@
         <v>1777</v>
       </c>
       <c r="X450" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="451" spans="1:24">
@@ -39070,7 +39088,7 @@
         <v>1777</v>
       </c>
       <c r="X451" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="452" spans="1:24">
@@ -39144,7 +39162,7 @@
         <v>1775</v>
       </c>
       <c r="X452" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="453" spans="1:24">
@@ -39218,7 +39236,7 @@
         <v>1777</v>
       </c>
       <c r="X453" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="454" spans="1:24">
@@ -39292,7 +39310,7 @@
         <v>1775</v>
       </c>
       <c r="X454" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="455" spans="1:24">
@@ -39366,7 +39384,7 @@
         <v>1777</v>
       </c>
       <c r="X455" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="456" spans="1:24">
@@ -39440,7 +39458,7 @@
         <v>1777</v>
       </c>
       <c r="X456" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="457" spans="1:24">
@@ -39514,7 +39532,7 @@
         <v>1775</v>
       </c>
       <c r="X457" t="s">
-        <v>1779</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="458" spans="1:24">
@@ -39588,7 +39606,7 @@
         <v>1777</v>
       </c>
       <c r="X458" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="459" spans="1:24">
@@ -39662,7 +39680,7 @@
         <v>1776</v>
       </c>
       <c r="X459" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="460" spans="1:24">
@@ -39736,7 +39754,7 @@
         <v>1775</v>
       </c>
       <c r="X460" t="s">
-        <v>1779</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="461" spans="1:24">
@@ -39810,7 +39828,7 @@
         <v>1777</v>
       </c>
       <c r="X461" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="462" spans="1:24">
@@ -39884,7 +39902,7 @@
         <v>1775</v>
       </c>
       <c r="X462" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="463" spans="1:24">
@@ -39958,7 +39976,7 @@
         <v>1775</v>
       </c>
       <c r="X463" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="464" spans="1:24">
@@ -40032,7 +40050,7 @@
         <v>1776</v>
       </c>
       <c r="X464" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="465" spans="1:24">
@@ -40106,7 +40124,7 @@
         <v>1775</v>
       </c>
       <c r="X465" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="466" spans="1:24">
@@ -40180,7 +40198,7 @@
         <v>1775</v>
       </c>
       <c r="X466" t="s">
-        <v>1779</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="467" spans="1:24">
@@ -40254,7 +40272,7 @@
         <v>1775</v>
       </c>
       <c r="X467" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="468" spans="1:24">
@@ -40328,7 +40346,7 @@
         <v>1775</v>
       </c>
       <c r="X468" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="469" spans="1:24">
@@ -40402,7 +40420,7 @@
         <v>1776</v>
       </c>
       <c r="X469" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="470" spans="1:24">
@@ -40476,7 +40494,7 @@
         <v>1777</v>
       </c>
       <c r="X470" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="471" spans="1:24">
@@ -40550,7 +40568,7 @@
         <v>1777</v>
       </c>
       <c r="X471" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="472" spans="1:24">
@@ -40624,7 +40642,7 @@
         <v>1777</v>
       </c>
       <c r="X472" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="473" spans="1:24">
@@ -40698,7 +40716,7 @@
         <v>1777</v>
       </c>
       <c r="X473" t="s">
-        <v>1789</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="474" spans="1:24">
@@ -40772,7 +40790,7 @@
         <v>1777</v>
       </c>
       <c r="X474" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="475" spans="1:24">
@@ -40846,7 +40864,7 @@
         <v>1775</v>
       </c>
       <c r="X475" t="s">
-        <v>1779</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="476" spans="1:24">
@@ -40920,7 +40938,7 @@
         <v>1777</v>
       </c>
       <c r="X476" t="s">
-        <v>1787</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="477" spans="1:24">
@@ -40994,7 +41012,7 @@
         <v>1775</v>
       </c>
       <c r="X477" t="s">
-        <v>1779</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="478" spans="1:24">
@@ -41068,7 +41086,7 @@
         <v>1776</v>
       </c>
       <c r="X478" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="479" spans="1:24">
@@ -41142,7 +41160,7 @@
         <v>1776</v>
       </c>
       <c r="X479" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="480" spans="1:24">
@@ -41216,7 +41234,7 @@
         <v>1776</v>
       </c>
       <c r="X480" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="481" spans="1:24">
@@ -41290,7 +41308,7 @@
         <v>1776</v>
       </c>
       <c r="X481" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="482" spans="1:24">
@@ -41364,7 +41382,7 @@
         <v>1777</v>
       </c>
       <c r="X482" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="483" spans="1:24">
@@ -41438,7 +41456,7 @@
         <v>1776</v>
       </c>
       <c r="X483" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="484" spans="1:24">
@@ -41512,7 +41530,7 @@
         <v>1775</v>
       </c>
       <c r="X484" t="s">
-        <v>1779</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="485" spans="1:24">
@@ -41586,7 +41604,7 @@
         <v>1775</v>
       </c>
       <c r="X485" t="s">
-        <v>1779</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="486" spans="1:24">
@@ -41660,7 +41678,7 @@
         <v>1775</v>
       </c>
       <c r="X486" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="487" spans="1:24">
@@ -41734,7 +41752,7 @@
         <v>1777</v>
       </c>
       <c r="X487" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="488" spans="1:24">
@@ -41808,7 +41826,7 @@
         <v>1776</v>
       </c>
       <c r="X488" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="489" spans="1:24">
@@ -41879,7 +41897,7 @@
         <v>1775</v>
       </c>
       <c r="X489" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="490" spans="1:24">
@@ -41953,7 +41971,7 @@
         <v>1776</v>
       </c>
       <c r="X490" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="491" spans="1:24">
@@ -42024,7 +42042,7 @@
         <v>1775</v>
       </c>
       <c r="X491" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="492" spans="1:24">
@@ -42095,7 +42113,7 @@
         <v>1776</v>
       </c>
       <c r="X492" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="493" spans="1:24">
@@ -42169,7 +42187,7 @@
         <v>1775</v>
       </c>
       <c r="X493" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="494" spans="1:24">
@@ -42240,7 +42258,7 @@
         <v>1776</v>
       </c>
       <c r="X494" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="495" spans="1:24">
@@ -42311,7 +42329,7 @@
         <v>1777</v>
       </c>
       <c r="X495" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="496" spans="1:24">
@@ -42385,7 +42403,7 @@
         <v>1778</v>
       </c>
       <c r="X496" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="497" spans="1:24">
@@ -42459,7 +42477,7 @@
         <v>1775</v>
       </c>
       <c r="X497" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="498" spans="1:24">
@@ -42533,7 +42551,7 @@
         <v>1777</v>
       </c>
       <c r="X498" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="499" spans="1:24">
@@ -42607,7 +42625,7 @@
         <v>1776</v>
       </c>
       <c r="X499" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="500" spans="1:24">
@@ -42681,7 +42699,7 @@
         <v>1776</v>
       </c>
       <c r="X500" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="501" spans="1:24">
@@ -42755,7 +42773,7 @@
         <v>1776</v>
       </c>
       <c r="X501" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="502" spans="1:24">
@@ -42829,7 +42847,7 @@
         <v>1776</v>
       </c>
       <c r="X502" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="503" spans="1:24">
@@ -42903,7 +42921,7 @@
         <v>1777</v>
       </c>
       <c r="X503" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="504" spans="1:24">
@@ -42974,7 +42992,7 @@
         <v>1777</v>
       </c>
       <c r="X504" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="505" spans="1:24">
@@ -43045,7 +43063,7 @@
         <v>1775</v>
       </c>
       <c r="X505" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="506" spans="1:24">
@@ -43119,7 +43137,7 @@
         <v>1776</v>
       </c>
       <c r="X506" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="507" spans="1:24">
@@ -43193,7 +43211,7 @@
         <v>1775</v>
       </c>
       <c r="X507" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="508" spans="1:24">
@@ -43267,7 +43285,7 @@
         <v>1775</v>
       </c>
       <c r="X508" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="509" spans="1:24">
@@ -43341,7 +43359,7 @@
         <v>1775</v>
       </c>
       <c r="X509" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="510" spans="1:24">
@@ -43415,7 +43433,7 @@
         <v>1776</v>
       </c>
       <c r="X510" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="511" spans="1:24">
@@ -43486,7 +43504,7 @@
         <v>1776</v>
       </c>
       <c r="X511" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="512" spans="1:24">
@@ -43557,7 +43575,7 @@
         <v>1776</v>
       </c>
       <c r="X512" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="513" spans="1:24">
@@ -43631,7 +43649,7 @@
         <v>1776</v>
       </c>
       <c r="X513" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="514" spans="1:24">
@@ -43705,7 +43723,7 @@
         <v>1776</v>
       </c>
       <c r="X514" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="515" spans="1:24">
@@ -43779,7 +43797,7 @@
         <v>1776</v>
       </c>
       <c r="X515" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="516" spans="1:24">
@@ -43850,7 +43868,7 @@
         <v>1776</v>
       </c>
       <c r="X516" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="517" spans="1:24">
@@ -43924,7 +43942,7 @@
         <v>1776</v>
       </c>
       <c r="X517" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="518" spans="1:24">
@@ -43995,7 +44013,7 @@
         <v>1776</v>
       </c>
       <c r="X518" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="519" spans="1:24">
@@ -44069,7 +44087,7 @@
         <v>1776</v>
       </c>
       <c r="X519" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="520" spans="1:24">
@@ -44143,7 +44161,7 @@
         <v>1776</v>
       </c>
       <c r="X520" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="521" spans="1:24">
@@ -44217,7 +44235,7 @@
         <v>1777</v>
       </c>
       <c r="X521" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="522" spans="1:24">
@@ -44291,7 +44309,7 @@
         <v>1776</v>
       </c>
       <c r="X522" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="523" spans="1:24">
@@ -44362,7 +44380,7 @@
         <v>1775</v>
       </c>
       <c r="X523" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="524" spans="1:24">
@@ -44436,7 +44454,7 @@
         <v>1776</v>
       </c>
       <c r="X524" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="525" spans="1:24">
@@ -44510,7 +44528,7 @@
         <v>1775</v>
       </c>
       <c r="X525" t="s">
-        <v>1779</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="526" spans="1:24">
@@ -44584,7 +44602,7 @@
         <v>1777</v>
       </c>
       <c r="X526" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="527" spans="1:24">
@@ -44658,7 +44676,7 @@
         <v>1776</v>
       </c>
       <c r="X527" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="528" spans="1:24">
@@ -44732,7 +44750,7 @@
         <v>1775</v>
       </c>
       <c r="X528" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="529" spans="1:24">
@@ -44806,7 +44824,7 @@
         <v>1776</v>
       </c>
       <c r="X529" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="530" spans="1:24">
@@ -44880,7 +44898,7 @@
         <v>1776</v>
       </c>
       <c r="X530" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="531" spans="1:24">
@@ -44954,7 +44972,7 @@
         <v>1777</v>
       </c>
       <c r="X531" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="532" spans="1:24">
@@ -45028,7 +45046,7 @@
         <v>1776</v>
       </c>
       <c r="X532" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="533" spans="1:24">
@@ -45102,7 +45120,7 @@
         <v>1777</v>
       </c>
       <c r="X533" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="534" spans="1:24">
@@ -45176,7 +45194,7 @@
         <v>1777</v>
       </c>
       <c r="X534" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="535" spans="1:24">
@@ -45250,7 +45268,7 @@
         <v>1777</v>
       </c>
       <c r="X535" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="536" spans="1:24">
@@ -45324,7 +45342,7 @@
         <v>1776</v>
       </c>
       <c r="X536" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="537" spans="1:24">
@@ -45395,7 +45413,7 @@
         <v>1775</v>
       </c>
       <c r="X537" t="s">
-        <v>1779</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="538" spans="1:24">
@@ -45469,7 +45487,7 @@
         <v>1776</v>
       </c>
       <c r="X538" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="539" spans="1:24">
@@ -45543,7 +45561,7 @@
         <v>1776</v>
       </c>
       <c r="X539" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="540" spans="1:24">
@@ -45617,7 +45635,7 @@
         <v>1776</v>
       </c>
       <c r="X540" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="541" spans="1:24">
@@ -45691,7 +45709,7 @@
         <v>1777</v>
       </c>
       <c r="X541" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="542" spans="1:24">
@@ -45762,7 +45780,7 @@
         <v>1776</v>
       </c>
       <c r="X542" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="543" spans="1:24">
@@ -45833,7 +45851,7 @@
         <v>1777</v>
       </c>
       <c r="X543" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="544" spans="1:24">
@@ -45907,7 +45925,7 @@
         <v>1777</v>
       </c>
       <c r="X544" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="545" spans="1:24">
@@ -45981,7 +45999,7 @@
         <v>1776</v>
       </c>
       <c r="X545" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="546" spans="1:24">
@@ -46055,7 +46073,7 @@
         <v>1776</v>
       </c>
       <c r="X546" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="547" spans="1:24">
@@ -46129,7 +46147,7 @@
         <v>1776</v>
       </c>
       <c r="X547" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="548" spans="1:24">
@@ -46203,7 +46221,7 @@
         <v>1776</v>
       </c>
       <c r="X548" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="549" spans="1:24">
@@ -46277,7 +46295,7 @@
         <v>1776</v>
       </c>
       <c r="X549" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="550" spans="1:24">
@@ -46351,7 +46369,7 @@
         <v>1776</v>
       </c>
       <c r="X550" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="551" spans="1:24">
@@ -46425,7 +46443,7 @@
         <v>1776</v>
       </c>
       <c r="X551" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="552" spans="1:24">
@@ -46499,7 +46517,7 @@
         <v>1776</v>
       </c>
       <c r="X552" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="553" spans="1:24">
@@ -46573,7 +46591,7 @@
         <v>1776</v>
       </c>
       <c r="X553" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="554" spans="1:24">
@@ -46647,7 +46665,7 @@
         <v>1776</v>
       </c>
       <c r="X554" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="555" spans="1:24">
@@ -46721,7 +46739,7 @@
         <v>1776</v>
       </c>
       <c r="X555" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="556" spans="1:24">
@@ -46795,7 +46813,7 @@
         <v>1776</v>
       </c>
       <c r="X556" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="557" spans="1:24">
@@ -46869,7 +46887,7 @@
         <v>1776</v>
       </c>
       <c r="X557" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="558" spans="1:24">
@@ -46943,7 +46961,7 @@
         <v>1776</v>
       </c>
       <c r="X558" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="559" spans="1:24">
@@ -47017,7 +47035,7 @@
         <v>1776</v>
       </c>
       <c r="X559" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="560" spans="1:24">
@@ -47091,7 +47109,7 @@
         <v>1776</v>
       </c>
       <c r="X560" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="561" spans="1:24">
@@ -47165,7 +47183,7 @@
         <v>1776</v>
       </c>
       <c r="X561" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="562" spans="1:24">
@@ -47239,7 +47257,7 @@
         <v>1776</v>
       </c>
       <c r="X562" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="563" spans="1:24">
@@ -47313,7 +47331,7 @@
         <v>1776</v>
       </c>
       <c r="X563" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
     </row>
   </sheetData>

</xml_diff>